<commit_message>
update some sheets, nerf some mp5 lowers
</commit_message>
<xml_diff>
--- a/changes/mp5.xlsx
+++ b/changes/mp5.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yifan/Documents/deadline-balancing/changes/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yifan\Documents\deadline-balancing\changes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1BC23CF-4C1A-C743-A6B7-E526A41ED9CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B12C3CB-0AE6-45F2-98F0-C2ACB950E544}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="18960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="m4-barrels" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
   <si>
     <t>new</t>
   </si>
@@ -126,13 +126,91 @@
   </si>
   <si>
     <t>HK MP5/HK94 Stock Endcap</t>
+  </si>
+  <si>
+    <t>hk_mp5_plastic_4_position_trigger_housing</t>
+  </si>
+  <si>
+    <t>HK MP5 Plastic 4 Position Trigger Housing</t>
+  </si>
+  <si>
+    <t>aeroknox_ax_mp5_trigger_housing</t>
+  </si>
+  <si>
+    <t>Aeroknox AX MP5 Trigger Housing</t>
+  </si>
+  <si>
+    <t>hk_mp5_sef_polymer_contoured_trigger_housing</t>
+  </si>
+  <si>
+    <t>HK MP5 SEF Polymer Contoured Trigger Housing</t>
+  </si>
+  <si>
+    <t>hk_mp5_hk94_sef_metal_trigger_housing</t>
+  </si>
+  <si>
+    <t>HK MP5/HK94 SEF Metal Trigger Housing</t>
+  </si>
+  <si>
+    <t>hk_mp5_wide_tropical_handguard</t>
+  </si>
+  <si>
+    <t>HK MP5 Wide Tropical</t>
+  </si>
+  <si>
+    <t>hk_mp5_slim_checkered_handguard</t>
+  </si>
+  <si>
+    <t>HK MP5 Slim Checkered Handguard</t>
+  </si>
+  <si>
+    <t>hk_mp5sd_polymer_handguard</t>
+  </si>
+  <si>
+    <t>HK MP5SD Polymer Handguard</t>
+  </si>
+  <si>
+    <t>bt_bt21343_3x_nar_mp5sd_handguard</t>
+  </si>
+  <si>
+    <t>B&amp;T BT-21343 3x NAR MP5SD Handguard</t>
+  </si>
+  <si>
+    <t>bt_bt401003_tl99_3x_nar_mp5_handguard</t>
+  </si>
+  <si>
+    <t>B&amp;T TL99 3x NAR MP5 Handguard</t>
+  </si>
+  <si>
+    <t>centrefire_628lmf_b_mp5_handguard</t>
+  </si>
+  <si>
+    <t>Surefire 628LMF-B MP5 Handguard</t>
+  </si>
+  <si>
+    <t>northeast_industries_mp5_mlok_handguard</t>
+  </si>
+  <si>
+    <t>Midwest Industries MP5 MLOK Handguard</t>
+  </si>
+  <si>
+    <t>ptr_mp5_trirail_handguard</t>
+  </si>
+  <si>
+    <t>PTR MP5 Trirail Handguard</t>
+  </si>
+  <si>
+    <t>tas_hx5_mp5_picatinny_handguard</t>
+  </si>
+  <si>
+    <t>CAA HX-5 MP5</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -266,6 +344,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="33">
@@ -609,8 +693,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -966,20 +1051,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:P27"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
-    <col min="2" max="2" width="33.83203125" customWidth="1"/>
-    <col min="3" max="22" width="6.6640625" customWidth="1"/>
+    <col min="2" max="2" width="33.85546875" customWidth="1"/>
+    <col min="3" max="22" width="6.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="C1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -1023,7 +1108,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>19</v>
       </c>
@@ -1046,11 +1131,11 @@
         <v>0</v>
       </c>
       <c r="N3">
-        <f t="shared" ref="N3:N12" si="0">C3-D3*20-E3*0.8-F3*0.6-H3*5+I3*10+J3/300</f>
+        <f t="shared" ref="N3:N27" si="0">C3-D3*20-E3*0.8-F3*0.6-H3*5+I3*10+J3/300</f>
         <v>18.2</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -1071,7 +1156,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -1098,7 +1183,7 @@
         <v>20.599999999999998</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -1119,7 +1204,7 @@
         <v>-1.4000000000000001</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>24</v>
       </c>
@@ -1140,7 +1225,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>25</v>
       </c>
@@ -1167,7 +1252,7 @@
         <v>20.8</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>22</v>
       </c>
@@ -1197,13 +1282,13 @@
         <v>-3.1999999999999993</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="N10">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>28</v>
       </c>
@@ -1256,7 +1341,7 @@
         <v>18.599999999999998</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>29</v>
       </c>
@@ -1307,6 +1392,407 @@
       <c r="N12">
         <f t="shared" si="0"/>
         <v>18.400000000000002</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C14" s="1">
+        <v>0</v>
+      </c>
+      <c r="D14" s="1">
+        <v>0.34</v>
+      </c>
+      <c r="E14" s="1">
+        <v>0</v>
+      </c>
+      <c r="F14" s="1">
+        <v>0</v>
+      </c>
+      <c r="G14" s="1"/>
+      <c r="H14" s="1"/>
+      <c r="I14" s="1"/>
+      <c r="J14" s="1"/>
+      <c r="K14" s="1"/>
+      <c r="L14" s="1"/>
+      <c r="M14" s="1">
+        <v>0</v>
+      </c>
+      <c r="N14">
+        <f t="shared" si="0"/>
+        <v>-6.8000000000000007</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C15" s="1">
+        <v>-4</v>
+      </c>
+      <c r="D15" s="1">
+        <v>0.32</v>
+      </c>
+      <c r="E15" s="1">
+        <v>3</v>
+      </c>
+      <c r="F15" s="1">
+        <v>3</v>
+      </c>
+      <c r="G15" s="1"/>
+      <c r="H15" s="1"/>
+      <c r="I15" s="1"/>
+      <c r="J15" s="1"/>
+      <c r="K15" s="1"/>
+      <c r="L15" s="1"/>
+      <c r="M15" s="1">
+        <v>1000</v>
+      </c>
+      <c r="N15">
+        <f t="shared" si="0"/>
+        <v>-14.600000000000001</v>
+      </c>
+      <c r="O15">
+        <f>N15+P15</f>
+        <v>-4.8000000000000007</v>
+      </c>
+      <c r="P15">
+        <v>9.8000000000000007</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C16" s="1">
+        <v>2</v>
+      </c>
+      <c r="D16" s="1">
+        <v>0.3</v>
+      </c>
+      <c r="E16" s="1">
+        <v>0</v>
+      </c>
+      <c r="F16" s="1">
+        <v>1</v>
+      </c>
+      <c r="G16" s="1"/>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
+      <c r="J16" s="1"/>
+      <c r="K16" s="1"/>
+      <c r="L16" s="1"/>
+      <c r="M16" s="1">
+        <v>1500</v>
+      </c>
+      <c r="N16">
+        <f t="shared" si="0"/>
+        <v>-4.5999999999999996</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C17" s="1">
+        <v>-1</v>
+      </c>
+      <c r="D17" s="1">
+        <v>0.34</v>
+      </c>
+      <c r="E17" s="1">
+        <v>2</v>
+      </c>
+      <c r="F17" s="1">
+        <v>4</v>
+      </c>
+      <c r="G17" s="1"/>
+      <c r="H17" s="1"/>
+      <c r="I17" s="1"/>
+      <c r="J17" s="1"/>
+      <c r="K17" s="1"/>
+      <c r="L17" s="1"/>
+      <c r="M17" s="1">
+        <v>1750</v>
+      </c>
+      <c r="N17">
+        <f t="shared" si="0"/>
+        <v>-11.8</v>
+      </c>
+      <c r="O17">
+        <f>N17+P17</f>
+        <v>-4.6000000000000005</v>
+      </c>
+      <c r="P17">
+        <v>7.2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N18">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>39</v>
+      </c>
+      <c r="B19" t="s">
+        <v>40</v>
+      </c>
+      <c r="C19">
+        <v>9</v>
+      </c>
+      <c r="D19">
+        <v>0.17</v>
+      </c>
+      <c r="E19">
+        <v>-10</v>
+      </c>
+      <c r="F19">
+        <v>-10</v>
+      </c>
+      <c r="M19">
+        <v>0</v>
+      </c>
+      <c r="N19">
+        <f t="shared" si="0"/>
+        <v>19.600000000000001</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>41</v>
+      </c>
+      <c r="B20" t="s">
+        <v>42</v>
+      </c>
+      <c r="C20">
+        <v>13</v>
+      </c>
+      <c r="D20">
+        <v>0.15</v>
+      </c>
+      <c r="E20">
+        <v>-7</v>
+      </c>
+      <c r="F20">
+        <v>-6</v>
+      </c>
+      <c r="M20">
+        <v>1500</v>
+      </c>
+      <c r="N20">
+        <f t="shared" si="0"/>
+        <v>19.200000000000003</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>43</v>
+      </c>
+      <c r="B21" t="s">
+        <v>44</v>
+      </c>
+      <c r="C21">
+        <v>11</v>
+      </c>
+      <c r="D21">
+        <v>0.16</v>
+      </c>
+      <c r="E21">
+        <v>-7</v>
+      </c>
+      <c r="F21">
+        <v>-8</v>
+      </c>
+      <c r="M21">
+        <v>1000</v>
+      </c>
+      <c r="N21">
+        <f t="shared" si="0"/>
+        <v>18.2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>45</v>
+      </c>
+      <c r="B22" t="s">
+        <v>46</v>
+      </c>
+      <c r="C22">
+        <v>7</v>
+      </c>
+      <c r="D22">
+        <v>0.22</v>
+      </c>
+      <c r="E22">
+        <v>-6</v>
+      </c>
+      <c r="F22">
+        <v>-7</v>
+      </c>
+      <c r="M22">
+        <v>1200</v>
+      </c>
+      <c r="N22">
+        <f t="shared" si="0"/>
+        <v>11.600000000000001</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>47</v>
+      </c>
+      <c r="B23" t="s">
+        <v>48</v>
+      </c>
+      <c r="C23">
+        <v>8</v>
+      </c>
+      <c r="D23">
+        <v>0.16</v>
+      </c>
+      <c r="E23">
+        <v>-6</v>
+      </c>
+      <c r="F23">
+        <v>-8</v>
+      </c>
+      <c r="M23">
+        <v>600</v>
+      </c>
+      <c r="N23">
+        <f t="shared" si="0"/>
+        <v>14.400000000000002</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>49</v>
+      </c>
+      <c r="B24" t="s">
+        <v>50</v>
+      </c>
+      <c r="C24">
+        <v>8</v>
+      </c>
+      <c r="D24">
+        <v>0.2</v>
+      </c>
+      <c r="E24">
+        <v>-9</v>
+      </c>
+      <c r="F24">
+        <v>-9</v>
+      </c>
+      <c r="M24">
+        <v>1200</v>
+      </c>
+      <c r="N24">
+        <f t="shared" si="0"/>
+        <v>16.599999999999998</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>51</v>
+      </c>
+      <c r="B25" t="s">
+        <v>52</v>
+      </c>
+      <c r="C25">
+        <v>9</v>
+      </c>
+      <c r="D25">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="E25">
+        <v>-6</v>
+      </c>
+      <c r="F25">
+        <v>-7</v>
+      </c>
+      <c r="M25">
+        <v>1000</v>
+      </c>
+      <c r="N25">
+        <f t="shared" si="0"/>
+        <v>15.2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>53</v>
+      </c>
+      <c r="B26" t="s">
+        <v>54</v>
+      </c>
+      <c r="C26">
+        <v>7</v>
+      </c>
+      <c r="D26">
+        <v>0.11</v>
+      </c>
+      <c r="E26">
+        <v>-8</v>
+      </c>
+      <c r="F26">
+        <v>-6</v>
+      </c>
+      <c r="M26">
+        <v>900</v>
+      </c>
+      <c r="N26">
+        <f t="shared" si="0"/>
+        <v>14.799999999999999</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>55</v>
+      </c>
+      <c r="B27" t="s">
+        <v>56</v>
+      </c>
+      <c r="C27">
+        <v>8</v>
+      </c>
+      <c r="D27">
+        <v>0.18</v>
+      </c>
+      <c r="E27">
+        <v>-7</v>
+      </c>
+      <c r="F27">
+        <v>-6</v>
+      </c>
+      <c r="M27">
+        <v>2500</v>
+      </c>
+      <c r="N27">
+        <f t="shared" si="0"/>
+        <v>13.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>